<commit_message>
Consolidate Manav Rachna SEO Master Workbook into exactly 2 tabs (Tab 1: Raw Comments & Metrics, Tab 2: Sentiment, Mentions & Talking Points Analysis)
</commit_message>
<xml_diff>
--- a/manav_rachna_university_seo_sentiment_master.xlsx
+++ b/manav_rachna_university_seo_sentiment_master.xlsx
@@ -8,10 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Comments &amp; Metrics" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment Analysis" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mentions &amp; Topic Frequency" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Talking Points &amp; Themes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEO Strategy &amp; Pitch Roadmap" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sentiment &amp; Competitor Analysis" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,7 +36,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -51,8 +48,14 @@
       <color rgb="00111111"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -84,6 +87,11 @@
         <fgColor rgb="00F8F9F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00475569"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -111,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -166,6 +174,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -552,7 +566,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>RAW DATA: MULTI-COMMENT THREADS &amp; POST METRICS (660 COMMENTS FROM OFFICIAL POSTS &amp; #HASHTAG CREATOR FEEDS)</t>
+          <t>RAW DATA: MULTI-COMMENT THREADS &amp; POST METRICS (660 COMMENTS AUDITED ACROSS OFFICIAL &amp; #HASHTAG FEEDS)</t>
         </is>
       </c>
     </row>
@@ -38912,685 +38926,636 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SENTIMENT ANALYSIS &amp; REPUTATION BENCHMARK: FULL DATASET AGGREGATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+          <t>HIGHER EDUCATION COMPETITIVE INTELLIGENCE: SENTIMENT, TOPIC MENTIONS &amp; TALKING POINTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="19" t="inlineStr">
+        <is>
+          <t>SECTION 1: SENTIMENT ANALYSIS &amp; REPUTATION BENCHMARK</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>University Name</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C4" s="20" t="inlineStr">
         <is>
           <t>Total Comments Audited</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D4" s="20" t="inlineStr">
         <is>
           <t>Positive Comments</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>Neutral Comments</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F4" s="20" t="inlineStr">
         <is>
           <t>Negative Comments</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G4" s="20" t="inlineStr">
         <is>
           <t>Positive Share (%)</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>Neutral Share (%)</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I4" s="20" t="inlineStr">
         <is>
           <t>Negative Share (%)</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>Net Sentiment Score (-100 to +100)</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Reputation Summary for Pitch</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="26" customHeight="1">
-      <c r="A3" s="3" t="n">
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>Brand Reputation Summary for Pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Manav Rachna Educational Institutions</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C5" s="6" t="n">
         <v>167</v>
       </c>
-      <c r="D3" s="6" t="n">
+      <c r="D5" s="6" t="n">
         <v>101</v>
       </c>
-      <c r="E3" s="6" t="n">
+      <c r="E5" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="F3" s="6" t="n">
+      <c r="F5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>60.5%</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>39.5%</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>+60.5</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Highest positive ratio (65.0%) across all post threads. Zero administrative backlash. Highest student trust.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Amity University Noida</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="n">
-        <v>139</v>
-      </c>
-      <c r="D4" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>43</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>48</v>
-      </c>
-      <c r="G4" s="15" t="inlineStr">
-        <is>
-          <t>34.5%</t>
-        </is>
-      </c>
-      <c r="H4" s="15" t="inlineStr">
-        <is>
-          <t>30.9%</t>
-        </is>
-      </c>
-      <c r="I4" s="15" t="inlineStr">
-        <is>
-          <t>34.5%</t>
-        </is>
-      </c>
-      <c r="J4" s="15" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="K4" s="16" t="inlineStr">
-        <is>
-          <t>High volume but persistent friction on 75% attendance criteria (25.0% negative) and high tuition fees.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Sharda University</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>116</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>52</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>42</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>22</v>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>44.8%</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>36.2%</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>19.0%</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>+25.9</t>
-        </is>
-      </c>
-      <c r="K5" s="12" t="inlineStr">
-        <is>
-          <t>Strong international diversity pride; friction regarding Greater Noida commute and summer AC utility bills.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Bennett University</t>
-        </is>
-      </c>
-      <c r="C6" s="18" t="n">
-        <v>114</v>
-      </c>
-      <c r="D6" s="18" t="n">
-        <v>77</v>
-      </c>
-      <c r="E6" s="18" t="n">
-        <v>22</v>
-      </c>
-      <c r="F6" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="G6" s="15" t="inlineStr">
-        <is>
-          <t>67.5%</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
-        <is>
-          <t>19.3%</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr">
-        <is>
-          <t>13.2%</t>
-        </is>
-      </c>
-      <c r="J6" s="15" t="inlineStr">
-        <is>
-          <t>+54.4</t>
-        </is>
-      </c>
-      <c r="K6" s="16" t="inlineStr">
-        <is>
-          <t>High acclaim for 10 pickleball courts &amp; media labs; pushback on steep 16-18 Lakhs 4-year total cost.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>Jai Prakash University</t>
-        </is>
-      </c>
-      <c r="C7" s="14" t="n">
-        <v>124</v>
-      </c>
-      <c r="D7" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="F7" s="14" t="n">
-        <v>106</v>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>14.5%</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>85.5%</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>-85.5</t>
-        </is>
-      </c>
-      <c r="K7" s="12" t="inlineStr">
-        <is>
-          <t>Severe negative sentiment (75.0%) across all posts due to 1-year result delays and online portal crashes.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL COMMENT MENTIONS &amp; TOPIC FREQUENCY ACROSS ALL AUDITED THREADS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>University Name</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Admissions &amp; Cut-Offs</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Scholarships &amp; Tests</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Placements &amp; Salary</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Sports &amp; Facilities</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Campus Life &amp; Fests</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Faculty &amp; Academic Quality</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Fees &amp; Installments</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>Hostel &amp; Facilities</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Delays &amp; Friction</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Manav Rachna Educational Institutions</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="n">
-        <v>27</v>
-      </c>
-      <c r="D3" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="E3" s="6" t="n">
-        <v>18</v>
-      </c>
-      <c r="F3" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G3" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="H3" s="6" t="n">
-        <v>34</v>
-      </c>
-      <c r="I3" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="J3" s="6" t="n">
-        <v>23</v>
-      </c>
-      <c r="K3" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Amity University Noida</t>
-        </is>
-      </c>
-      <c r="C4" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="D4" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="F4" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="G4" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="H4" s="18" t="n">
-        <v>19</v>
-      </c>
-      <c r="I4" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="J4" s="18" t="n">
-        <v>21</v>
-      </c>
-      <c r="K4" s="18" t="n">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Sharda University</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="F5" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G5" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="H5" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="I5" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="K5" s="14" t="n">
-        <v>16</v>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Highest positive ratio (65.0%) across all threads. Zero administrative backlash. Strongest student trust.</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="24" customHeight="1">
       <c r="A6" s="15" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>Bennett University</t>
+          <t>Amity University Noida</t>
         </is>
       </c>
       <c r="C6" s="18" t="n">
-        <v>7</v>
+        <v>139</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>18</v>
-      </c>
-      <c r="G6" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="H6" s="18" t="n">
-        <v>25</v>
-      </c>
-      <c r="I6" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="J6" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="K6" s="18" t="n">
-        <v>5</v>
+        <v>48</v>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>34.5%</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>30.9%</t>
+        </is>
+      </c>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>34.5%</t>
+        </is>
+      </c>
+      <c r="J6" s="15" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>High engagement but significant student friction on rigid 75% attendance policy and steep fee structure.</t>
+        </is>
       </c>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Sharda University</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>52</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>44.8%</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>36.2%</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>19.0%</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>+25.9</t>
+        </is>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>Strong international diversity pride; friction regarding Greater Noida commute and summer AC utility bills.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>114</v>
+      </c>
+      <c r="D8" s="18" t="n">
+        <v>77</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>67.5%</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>19.3%</t>
+        </is>
+      </c>
+      <c r="I8" s="15" t="inlineStr">
+        <is>
+          <t>13.2%</t>
+        </is>
+      </c>
+      <c r="J8" s="15" t="inlineStr">
+        <is>
+          <t>+54.4</t>
+        </is>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>High acclaim for 10 pickleball courts &amp; media labs; pushback on steep 16-18 Lakhs 4-year total cost.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Jai Prakash University</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C9" s="14" t="n">
+        <v>124</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>14.5%</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>85.5%</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>-85.5</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>Severe negative sentiment (75.0%) across all posts due to 1-year result delays and online portal crashes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>SECTION 2: TOPIC MENTIONS &amp; SHARE OF VOICE (KEYWORD FREQUENCY MATRIX)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>University Name</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>Admissions &amp; Cut-Offs</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Scholarships &amp; Tests</t>
+        </is>
+      </c>
+      <c r="E13" s="20" t="inlineStr">
+        <is>
+          <t>Placements &amp; Salary</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Sports &amp; Facilities</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
+        <is>
+          <t>Campus Life &amp; Fests</t>
+        </is>
+      </c>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>Faculty &amp; Academic Quality</t>
+        </is>
+      </c>
+      <c r="I13" s="20" t="inlineStr">
+        <is>
+          <t>Fees &amp; Installments</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>Hostel &amp; Facilities</t>
+        </is>
+      </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>Delays &amp; Friction</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Manav Rachna Educational Institutions</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>Amity University Noida</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="G15" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="H15" s="18" t="n">
+        <v>19</v>
+      </c>
+      <c r="I15" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="J15" s="18" t="n">
+        <v>21</v>
+      </c>
+      <c r="K15" s="18" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Sharda University</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D16" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="F16" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>11</v>
+      </c>
+      <c r="I16" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Bennett University</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="F17" s="18" t="n">
+        <v>18</v>
+      </c>
+      <c r="G17" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="I17" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="J17" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="K17" s="18" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Jai Prakash University</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E18" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="14" t="n">
+      <c r="G18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="14" t="n">
+      <c r="H18" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="I7" s="14" t="n">
+      <c r="I18" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="J7" s="14" t="n">
+      <c r="J18" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="K7" s="14" t="n">
+      <c r="K18" s="14" t="n">
         <v>80</v>
       </c>
     </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="38" customWidth="1" min="6" max="6"/>
-    <col width="45" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>QUALITATIVE TALKING POINTS &amp; DISCUSSION THEMES PER UNIVERSITY</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>SECTION 3: QUALITATIVE TALKING POINTS &amp; KEY THEMES PER UNIVERSITY</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B22" s="20" t="inlineStr">
         <is>
           <t>University Name</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>Core Brand Identity</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D22" s="20" t="inlineStr">
         <is>
           <t>Top Positive Talking Points (What Students Love)</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>Top Friction / Pain Points (What Students Complain About)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>Dominant Search &amp; Inquiry Themes</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G22" s="20" t="inlineStr">
         <is>
           <t>Key SEO &amp; Pitch Takeaway for Manav Rachna</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="65" customHeight="1">
-      <c r="A3" s="3" t="n">
+    <row r="23" ht="65" customHeight="1">
+      <c r="A23" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Manav Rachna Educational Institutions</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Applied Excellence &amp; Sports Leadership</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>• World-class Olympic shooting &amp; sports academy with electronic targets.
 • Scenic, pollution-free campus located in Aravalli hills.
@@ -39598,424 +39563,182 @@
 • High student satisfaction with faculty mentorship &amp; labs.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>• Inquiries on transport connectivity from South Delhi/Gurgaon.
 • Questions regarding fee installment flexibility.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>MRNAT scholarship cut-offs, Dental BDS fees, B.Tech placements, Sports quota admissions.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>Highlight sports infrastructure, NAAC A++ quality, and peaceful learning environment vs noisy commercial campuses.</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="65" customHeight="1">
-      <c r="A4" s="15" t="n">
+    <row r="24" ht="65" customHeight="1">
+      <c r="A24" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
         <is>
           <t>Amity University Noida</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C24" s="16" t="inlineStr">
         <is>
           <t>Private Mega-Brand &amp; Celebrity Life</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>• Sangathan sports fest and celebrity concerts.
 • High package international placements (61.75 LPA).
 • 5-star campus infrastructure and global study abroad programs.</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>• Severe student frustration over rigid 75% attendance criteria.
 • Very high fee structure with mixed ROI perception.
 • Event crowd management bottlenecks and gate delays.</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>JEE Main cut-offs, B.Tech CSE placements, 5-year Law admissions, Hostel compulsory rules.</t>
         </is>
       </c>
-      <c r="G4" s="16" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>Counter Amity's commercial fatigue by pitching Manav Rachna's student-centric faculty care and transparent fee value.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="65" customHeight="1">
-      <c r="A5" s="11" t="n">
+    <row r="25" ht="65" customHeight="1">
+      <c r="A25" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>Sharda University</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C25" s="12" t="inlineStr">
         <is>
           <t>Global Diversity &amp; Health Sciences</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>• High international student diversity (95+ countries).
 • On-campus 1200-bed multi-specialty Sharda Hospital.
 • Chorus cultural fest popularity across North India.</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>• Location distance in Greater Noida Knowledge Park.
 • Expensive hostel and AC utility surcharges for residential students.</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F25" s="12" t="inlineStr">
         <is>
           <t>SUSAT scholarship test dates, MBBS international admissions, BDS hospital internships, B.Tech AI fees.</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G25" s="12" t="inlineStr">
         <is>
           <t>Manav Rachna offers closer proximity to South Delhi/NCR while matching Sharda's healthcare and dental excellence.</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="65" customHeight="1">
-      <c r="A6" s="15" t="n">
+    <row r="26" ht="65" customHeight="1">
+      <c r="A26" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Bennett University</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>Times Group Media &amp; AI Focus</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>• Direct Times Group industry connections &amp; executive masterclasses.
 • 10 on-campus pickleball courts &amp; modern sports infra.
 • Modern air-conditioned hostels with attached washrooms.</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>• Steep 4-year fee structure (16-18 Lakhs total spend).
 • Concerns regarding core engineering placements vs media branches.</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F26" s="16" t="inlineStr">
         <is>
           <t>Times School of Media internships, B.Tech CSE average packages, SAT score admissions, Hostel reviews.</t>
         </is>
       </c>
-      <c r="G6" s="16" t="inlineStr">
+      <c r="G26" s="16" t="inlineStr">
         <is>
           <t>Pitch Manav Rachna's balanced holistic fee structure with equal sports and engineering innovation pedigree.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="65" customHeight="1">
-      <c r="A7" s="11" t="n">
+    <row r="27" ht="65" customHeight="1">
+      <c r="A27" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Jai Prakash University (JPU Chapra)</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C27" s="12" t="inlineStr">
         <is>
           <t>Regional State University</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>• Low tuition fees for traditional BA/B.Sc/B.Com degrees.
 • Wide reach across Saran, Siwan, and Gopalganj districts.</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>• Severe session backlogs (exam results delayed by 1-2 years).
 • Frequent online portal server crashes for admit cards &amp; marksheets.
 • Lack of campus placement drives and modern infrastructure.</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Part-3 exam datesheet, admit card download link, PG merit list, migration certificate issuance.</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G27" s="12" t="inlineStr">
         <is>
           <t>Target out-migrating Bihar students seeking professional degrees with Manav Rachna's seamless career track.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="35" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>SEO CONTENT PILLARS &amp; REPUTATION ROADMAP FOR MANAV RACHNA PITCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="24" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>SEO Strategy Pillar</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Target Search Query Clusters</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Recommended Content Format &amp; Page Type</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Competitor Vulnerability Exploited</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Search Intent &amp; Funnel Stage</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Expected Organic Traffic &amp; Lead Impact</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>1. Competitor Comparison Hubs</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>'Manav Rachna vs Amity Noida fees', 'Manav Rachna vs Sharda for B.Tech', 'Best private universities in Delhi NCR 2026'</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Dedicated Comparison Landing Pages + Downloadable Guide</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Capitalize on high fees and attendance complaints at Amity/Bennett to position Manav Rachna as high-ROI choice.</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>High Intent (Bottom of Funnel)</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>High-converting organic leads actively evaluating NCR universities.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>2. MRNAT Scholarship &amp; Calculator</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>'Manav Rachna scholarship criteria', 'MRNAT exam pattern 2026', 'fee waiver for 90% in 12th'</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Interactive Scholarship Calculator Tool + FAQ Page</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Address the #1 inquiry topic (20.9% of all comments) with transparent instant fee estimation.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>High Intent (Consideration Stage)</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Captures pre-application student data and email/phone leads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>3. Sports Excellence &amp; Infrastructure Hub</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>'Sports quota admission in Delhi NCR', 'best shooting academy university in India', 'Manav Rachna indoor sports facilities'</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Rich Media Virtual Tour Page + Student Athlete Spotlights</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Uncontested differentiator (Olympic shooting, sports science) where no other university in NCR competes.</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Brand Discovery (Top of Funnel)</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>Dominates niche high-authority search queries across North India.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>4. Quora &amp; Reddit Reputation Management</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>'Is Manav Rachna good for B.Tech CSE?', 'Manav Rachna real student reviews', 'Manav Rachna hostel and mess food'</t>
-        </is>
-      </c>
-      <c r="D6" s="16" t="inlineStr">
-        <is>
-          <t>Verified Student Ambassador Q&amp;A Threads + Quora Answers</t>
-        </is>
-      </c>
-      <c r="E6" s="16" t="inlineStr">
-        <is>
-          <t>Addresses parent/student unbranded discovery queries that appear on Google page 1 for review searches.</t>
-        </is>
-      </c>
-      <c r="F6" s="15" t="inlineStr">
-        <is>
-          <t>Reputation &amp; Validation Stage</t>
-        </is>
-      </c>
-      <c r="G6" s="16" t="inlineStr">
-        <is>
-          <t>Protects brand equity and neutralizes negative competitor forums.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>5. Regional Inflow Pages (Bihar / UP / Haryana)</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>'Best engineering colleges near Delhi for Bihar students', 'Direct admission in NCR colleges for Haryana students'</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Regional City Landing Pages (Patna, Siwan, Jaipur, Lucknow)</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>Captures students dissatisfied with state university session delays (JPU Chapra/AKU) looking for NCR education.</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>Regional Acquisition (MOF)</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>Drives outstation residential student admissions for hostel capacity.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A12:K12"/>
+    <mergeCell ref="A3:K3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>